<commit_message>
Update Board 9 July and August hourly workbooks
</commit_message>
<xml_diff>
--- a/data/soil_data/matric_potential_conductivity/Berger Hourly Data Collection_Board_ID 9_2026-08-26.xlsx
+++ b/data/soil_data/matric_potential_conductivity/Berger Hourly Data Collection_Board_ID 9_2026-08-26.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e5e73ff6e8b2309b/Documents/SourceCode/Photo3-Plant-Salinity-Traits/data/soil_data/matric_potential_conductivity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_791153A6D390D05D3572D5734B5ED87656C91D37" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD896BE2-13FA-41B4-B746-E8F571E55566}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_791153A6D390D05D3572D5734B5ED87656C91D37" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{169A5C27-413A-4ED1-B584-02FEA0B4C88A}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="2205" windowWidth="16200" windowHeight="9307" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -126,7 +139,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -159,7 +172,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -175,6 +188,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -465,7 +482,10 @@
   <dimension ref="A1:AG168"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="24" max="24" width="14.265625" customWidth="1"/>
     <col min="27" max="27" width="14.46484375" customWidth="1"/>
+    <col min="31" max="31" width="14.3984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.45">
@@ -1460,7 +1480,7 @@
         <v>24.428888612323341</v>
       </c>
       <c r="AB10">
-        <v>2212.8780504014758</v>
+        <v>2212.8780504014799</v>
       </c>
       <c r="AC10">
         <v>24.059444671207</v>

</xml_diff>